<commit_message>
Add filled Room Profiles to new templates
47 rooms with capacity, available periods (A-G), available terms
(FY,S1,S2), and shared status. Note: J-322 appears twice with
different capacities (30 and 32) — preserved as uploaded.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/new/Template_9_Room_Profiles.xlsx
+++ b/templates/new/Template_9_Room_Profiles.xlsx
@@ -33,14 +33,13 @@
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00375623"/>
-      <sz val="10"/>
+      <b val="1"/>
+      <color rgb="00A63D2B"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00808080"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -52,14 +51,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5496"/>
-        <bgColor rgb="002F5496"/>
+        <fgColor rgb="001B4965"/>
+        <bgColor rgb="001B4965"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FDE8E4"/>
+        <bgColor rgb="00FDE8E4"/>
       </patternFill>
     </fill>
   </fills>
@@ -72,10 +71,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00D4D0C8"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D4D0C8"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D4D0C8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D4D0C8"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -84,7 +91,7 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -455,13 +462,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -522,7 +529,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>J-322</t>
+          <t>Auditorium</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
@@ -533,19 +540,1168 @@
           <t>A,B,C,D,E,F,G</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>D-101</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>D-102</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>D-103</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>D-104</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>D-105</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>D-106</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>D-107</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>D-108</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>D-109</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>D-110</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>D-201</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>D-202</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>D-203</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>D-204</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>D-205</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>D-206</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>D-210</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Gym</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>I-011</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>I-012</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>I-113</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>I-114</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>I-115</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>I-116</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>I-117</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>I-118</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>I-119</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>J-020</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>J-120</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>J-221</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>J-222</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>J-320</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>J-321</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>J-322</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>J-322</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>J-323</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>S-231</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>S-232</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>S-233</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>S-234</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>S-235</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>S-236</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>S-237</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>S-238</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>S-338</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Success Center</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>FY,S1,S2</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="E3:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Y/N" prompt="Enter Y or N" type="list">
-      <formula1>"Y,N"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>